<commit_message>
feat: align training schedule and countdowns with official ICPC 2026 & OLP'26 dates
</commit_message>
<xml_diff>
--- a/ICPC_OLP_Training_Deruck.xlsx
+++ b/ICPC_OLP_Training_Deruck.xlsx
@@ -591,7 +591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -649,124 +649,124 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>2026-10-17 (Thứ Bảy)</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Tuần 1: VÒNG THI ICPC MIỀN NAM 2026 &amp; Củng cố Cây (Tree), DSU</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Thử máy Vòng thi ICPC Miền Nam 2026 (ĐH KHTN TP.HCM)</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/gyms</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>ICPC Miền Nam 2026 - Practice Session</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>ICPC Team</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>THỬ MÁY</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-18 (Chủ Nhật)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Tuần 1: VÒNG THI ICPC MIỀN NAM 2026 &amp; Củng cố Cây (Tree), DSU</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>CHÍNH THỨC THI ICPC MIỀN NAM 2026 (5 GIỜ)</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/gyms</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>ICPC Southern Vietnam Regional Contest 2026</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>ICPC Team</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>OFFICIAL CONTEST</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
           <t>2026-10-19 (Thứ Hai)</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Tuần 1: Củng cố Cây (Tree), DSU nâng cao &amp; Đường đi ngắn nhất (Shortest Path)</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Ôn tập Lý thuyết &amp; Re-solve bài cũ: DSU Tree &amp; Small to Large</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>https://codeforces.com/contest/1416/problem/D</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Codeforces 1416D - DSU Tree</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>2600</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>Re-solve bài cũ</t>
-        </is>
-      </c>
-      <c r="H2" s="7" t="inlineStr">
-        <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-20 (Thứ Ba)</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Tuần 1: Củng cố Cây (Tree), DSU nâng cao &amp; Đường đi ngắn nhất (Shortest Path)</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Luyện tập Ladder 16: Graph &amp; Shortest Paths</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>https://codeforces.com/contest/295/problem/B</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Codeforces 295B - Greg and Graph (Floyd-Warshall trick)</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>1700</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>Ladder 16 Re-solve</t>
-        </is>
-      </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-21 (Thứ Tư)</t>
-        </is>
-      </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Tuần 1: Củng cố Cây (Tree), DSU nâng cao &amp; Đường đi ngắn nhất (Shortest Path)</t>
+          <t>Tuần 1: VÒNG THI ICPC MIỀN NAM 2026 &amp; Củng cố Cây (Tree), DSU</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Kiểm tra cá nhân OLP Mini-Contest #1 (2.5h)</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>https://codeforces.com/contest/1996</t>
-        </is>
-      </c>
-      <c r="E4" s="10" t="inlineStr">
-        <is>
-          <t>Codeforces Round 962 (Div. 3/2)</t>
+          <t>Upsolving đề ICPC Miền Nam &amp; Phân tích lỗi kỹ thuật phòng thi</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/gyms</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Upsolve ICPC Miền Nam</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>1200-1800</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>Mini Mock Test</t>
-        </is>
-      </c>
-      <c r="H4" s="11" t="inlineStr">
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Upsolving</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>Chưa làm</t>
         </is>
@@ -775,32 +775,32 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22 (Thứ Năm)</t>
+          <t>2026-10-20 (Thứ Ba)</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Tuần 1: Củng cố Cây (Tree), DSU nâng cao &amp; Đường đi ngắn nhất (Shortest Path)</t>
+          <t>Tuần 1: VÒNG THI ICPC MIỀN NAM 2026 &amp; Củng cố Cây (Tree), DSU</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Re-solve bài cũ: Mo on Tree &amp; Rerooting</t>
+          <t>Re-solve bài cũ: DSU Tree &amp; Small to Large</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/problemset/problem/375/D</t>
+          <t>https://codeforces.com/contest/1416/problem/D</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Codeforces 375D - Mo on tree</t>
+          <t>Codeforces 1416D - DSU Tree</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>2400</t>
+          <t>2600</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -817,37 +817,37 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23 (Thứ Sáu)</t>
+          <t>2026-10-21 (Thứ Tư)</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Tuần 1: Củng cố Cây (Tree), DSU nâng cao &amp; Đường đi ngắn nhất (Shortest Path)</t>
+          <t>Tuần 1: VÒNG THI ICPC MIỀN NAM 2026 &amp; Củng cố Cây (Tree), DSU</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Thực hành Ladder 16: DFS/BFS &amp; Constructive</t>
+          <t>Ladder 16 Re-solve: Graph &amp; Shortest Paths (Floyd trick)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/problemset/problem/217/A</t>
+          <t>https://codeforces.com/contest/295/problem/B</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Codeforces 217A - Ice Skating</t>
+          <t>Codeforces 295B - Greg and Graph</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>1400</t>
+          <t>1700</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Ladder 16</t>
+          <t>Ladder 16 Re-solve</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
@@ -859,37 +859,37 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24 (Thứ Bảy)</t>
+          <t>2026-10-22 (Thứ Năm)</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Tuần 1: Củng cố Cây (Tree), DSU nâng cao &amp; Đường đi ngắn nhất (Shortest Path)</t>
+          <t>Tuần 1: VÒNG THI ICPC MIỀN NAM 2026 &amp; Củng cố Cây (Tree), DSU</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Upsolving &amp; Tối ưu hóa Code Template (Tree/Graph)</t>
+          <t>Re-solve bài cũ: Mo on Tree &amp; Rerooting</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>https://oj.vnoi.info/problem/diffgraph</t>
+          <t>https://codeforces.com/problemset/problem/375/D</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>LQDOJ diffgraph - Small to large, reroot</t>
+          <t>Codeforces 375D - Mo on tree</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>2400</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>VNOI/LQDOJ Practice</t>
+          <t>Re-solve bài cũ</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
@@ -899,42 +899,42 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-25 (Chủ Nhật)</t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Tuần 1: Củng cố Cây (Tree), DSU nâng cao &amp; Đường đi ngắn nhất (Shortest Path)</t>
+          <t>Tuần 1: VÒNG THI ICPC MIỀN NAM 2026 &amp; Củng cố Cây (Tree), DSU</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>MOCK TEST 1: ICPC Regional Simulation 5 Giờ (Team Contest #1)</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>https://codeforces.com/gym/104021</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="inlineStr">
-        <is>
-          <t>2022-2023 ICPC Asia Yokohama Regional</t>
+          <t>Rà soát Template &amp; Chuẩn bị chiến thuật Vòng Miền Trung</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/problemset/problem/217/A</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Codeforces 217A - Ice Skating</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>ICPC Team</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>FULL MOCK TEST</t>
-        </is>
-      </c>
-      <c r="H8" s="11" t="inlineStr">
+          <t>1400</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Review Template</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>Chưa làm</t>
         </is>
@@ -943,37 +943,37 @@
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26 (Thứ Hai)</t>
+          <t>2026-10-24 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Tuần 2: Dynamic Programming nâng cao (SOS DP, CHT, Bitmask, Tree DP)</t>
+          <t>Tuần 2: VÒNG THI ICPC MIỀN TRUNG 2026 &amp; Quy hoạch động nâng cao (SOS DP, CHT)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Ôn tập SOS DP &amp; Bitmask: Re-solve các bài kinh điển</t>
+          <t>Thử máy Vòng thi ICPC Miền Trung 2026 (ĐH Khoa học - ĐH Huế)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>https://cses.fi/problemset/task/1654</t>
+          <t>https://codeforces.com/gyms</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>CSES 1654 - SOS DP</t>
+          <t>ICPC Miền Trung 2026 - Practice Session</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>2100</t>
+          <t>ICPC Team</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Re-solve</t>
+          <t>THỬ MÁY</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -983,42 +983,42 @@
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-27 (Thứ Ba)</t>
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-25 (Chủ Nhật)</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Tuần 2: Dynamic Programming nâng cao (SOS DP, CHT, Bitmask, Tree DP)</t>
+          <t>Tuần 2: VÒNG THI ICPC MIỀN TRUNG 2026 &amp; Quy hoạch động nâng cao (SOS DP, CHT)</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Re-solve bài cũ: SOS DP &amp; Bao hàm loại trừ</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>https://codeforces.com/problemset/problem/449/D</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Codeforces 449D - Jzzhu and Numbers</t>
+          <t>CHÍNH THỨC THI ICPC MIỀN TRUNG 2026 (5 GIỜ)</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/gyms</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>ICPC Central Vietnam Regional Contest 2026</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>2400</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Re-solve bài cũ</t>
-        </is>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
+          <t>ICPC Team</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>OFFICIAL CONTEST</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
         <is>
           <t>Chưa làm</t>
         </is>
@@ -1027,37 +1027,37 @@
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28 (Thứ Tư)</t>
+          <t>2026-10-26 (Thứ Hai)</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Tuần 2: Dynamic Programming nâng cao (SOS DP, CHT, Bitmask, Tree DP)</t>
+          <t>Tuần 2: VÒNG THI ICPC MIỀN TRUNG 2026 &amp; Quy hoạch động nâng cao (SOS DP, CHT)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Kiểm tra cá nhân OLP Mock Contest #2 (3h)</t>
+          <t>Upsolve đề Miền Trung &amp; Củng cố SOS DP</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/contest/1987</t>
+          <t>https://cses.fi/problemset/task/1654</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Codeforces Round 955 (Div. 2/1)</t>
+          <t>CSES 1654 - SOS DP</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>1500-2200</t>
+          <t>2100</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>OLP Mock Test</t>
+          <t>Re-solve bài cũ</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -1069,27 +1069,27 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29 (Thứ Năm)</t>
+          <t>2026-10-27 (Thứ Ba)</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Tuần 2: Dynamic Programming nâng cao (SOS DP, CHT, Bitmask, Tree DP)</t>
+          <t>Tuần 2: VÒNG THI ICPC MIỀN TRUNG 2026 &amp; Quy hoạch động nâng cao (SOS DP, CHT)</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Convex Hull Trick &amp; Li Chao Tree / Alien's Trick</t>
+          <t>Re-solve bài cũ: SOS DP &amp; Bao hàm loại trừ</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/problemset/problem/1715/E</t>
+          <t>https://codeforces.com/problemset/problem/449/D</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Codeforces 1715E - Long Way Home (Dijkstra + CHT)</t>
+          <t>Codeforces 449D - Jzzhu and Numbers</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -1109,42 +1109,42 @@
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-30 (Thứ Sáu)</t>
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-28 (Thứ Tư)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Tuần 2: Dynamic Programming nâng cao (SOS DP, CHT, Bitmask, Tree DP)</t>
+          <t>Tuần 2: VÒNG THI ICPC MIỀN TRUNG 2026 &amp; Quy hoạch động nâng cao (SOS DP, CHT)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Ladder 16: DP &amp; Strings (KMP + DP)</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>https://codeforces.com/problemset/problem/346/B</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Codeforces 346B - Lucky Common Subsequence</t>
+          <t>Kiểm tra cá nhân OLP Mini-Mock Contest (2.5h - CF Div.2)</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/contest/1987</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Codeforces Round 955 (Div. 2/1)</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Ladder 16 Re-solve</t>
-        </is>
-      </c>
-      <c r="H13" s="7" t="inlineStr">
+          <t>1500-2200</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>OLP Mini Test</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr">
         <is>
           <t>Chưa làm</t>
         </is>
@@ -1153,37 +1153,37 @@
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31 (Thứ Bảy)</t>
+          <t>2026-10-29 (Thứ Năm)</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Tuần 2: Dynamic Programming nâng cao (SOS DP, CHT, Bitmask, Tree DP)</t>
+          <t>Tuần 2: VÒNG THI ICPC MIỀN TRUNG 2026 &amp; Quy hoạch động nâng cao (SOS DP, CHT)</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Upsolve các bài DP chưa hoàn thành &amp; Team Strategy</t>
+          <t>Convex Hull Trick &amp; Li Chao Tree / Alien's Trick</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>https://oj.vnoi.info/problem/voi21_or</t>
+          <t>https://codeforces.com/problemset/problem/1715/E</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>VOI 2021 OR - SOS DP</t>
+          <t>Codeforces 1715E - Long Way Home (Dijkstra + CHT)</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>VOI</t>
+          <t>2400</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>VOI Practice</t>
+          <t>Re-solve bài cũ</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
@@ -1193,42 +1193,42 @@
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>2026-11-01 (Chủ Nhật)</t>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Tuần 2: Dynamic Programming nâng cao (SOS DP, CHT, Bitmask, Tree DP)</t>
+          <t>Tuần 2: VÒNG THI ICPC MIỀN TRUNG 2026 &amp; Quy hoạch động nâng cao (SOS DP, CHT)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>MOCK TEST 2: ICPC Regional Simulation 5 Giờ (Team Contest #2)</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>https://codeforces.com/gym/104114</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>2022 ICPC Asia Can Tho Regional Contest</t>
+          <t>Ladder 16 Re-solve: KMP + DP</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/problemset/problem/346/B</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Codeforces 346B - Lucky Common Subsequence</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>ICPC Team</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>FULL MOCK TEST</t>
-        </is>
-      </c>
-      <c r="H15" s="11" t="inlineStr">
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Ladder 16 Re-solve</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>Chưa làm</t>
         </is>
@@ -1237,12 +1237,12 @@
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-11-02 (Thứ Hai)</t>
+          <t>2026-10-31 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Tuần 3: Cấu trúc dữ liệu nâng cao &amp; Chia căn (Mo, Sqrt Decomposition, SegTree)</t>
+          <t>Tuần 3: TỔNG LỰC CHUẨN BỊ CHO KỲ THI ICPC QUỐC GIA 2026</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1279,37 +1279,37 @@
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-11-03 (Thứ Ba)</t>
+          <t>2026-11-01 (Chủ Nhật)</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Tuần 3: Cấu trúc dữ liệu nâng cao &amp; Chia căn (Mo, Sqrt Decomposition, SegTree)</t>
+          <t>Tuần 3: TỔNG LỰC CHUẨN BỊ CHO KỲ THI ICPC QUỐC GIA 2026</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Ladder 16: Segment Tree &amp; Modulo Trick</t>
+          <t>MOCK TEST QUỐC GIA 5H: Giả lập ICPC Vietnam National 2023</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/problemset/problem/438/D</t>
+          <t>https://codeforces.com/gym/104725</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Codeforces 438D - The Child and Sequence</t>
+          <t>2023 ICPC Vietnam National Contest</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>2300</t>
+          <t>ICPC Team</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Ladder 16 Re-solve</t>
+          <t>FULL MOCK TEST</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -1321,37 +1321,37 @@
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-11-04 (Thứ Tư)</t>
+          <t>2026-11-02 (Thứ Hai)</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Tuần 3: Cấu trúc dữ liệu nâng cao &amp; Chia căn (Mo, Sqrt Decomposition, SegTree)</t>
+          <t>Tuần 3: TỔNG LỰC CHUẨN BỊ CHO KỲ THI ICPC QUỐC GIA 2026</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Kiểm tra cá nhân OLP Mock Contest #3 (3.5h - CTDL &amp; DP)</t>
+          <t>Upsolve đề Mock Test Quốc Gia &amp; Tối ưu hóa phân chia bài</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>https://oj.vnoi.info/problem/coci1920_o_paint</t>
+          <t>https://codeforces.com/problemset/problem/438/D</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>COCI 1920 Paint - Chia căn lớn bé &amp; DSU</t>
+          <t>Codeforces 438D - The Child and Sequence (SegTree Modulo)</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>2300</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>OLP Mock Test</t>
+          <t>Upsolving</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
@@ -1363,37 +1363,37 @@
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-11-05 (Thứ Năm)</t>
+          <t>2026-11-03 (Thứ Ba)</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Tuần 3: Cấu trúc dữ liệu nâng cao &amp; Chia căn (Mo, Sqrt Decomposition, SegTree)</t>
+          <t>Tuần 3: TỔNG LỰC CHUẨN BỊ CHO KỲ THI ICPC QUỐC GIA 2026</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Persistent Segment Tree &amp; Treap cơ bản</t>
+          <t>Kiểm tra và in ấn Team Notebook bản chuẩn cho kỳ thi Quốc Gia</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/contest/986/problem/E</t>
+          <t>https://codeforces.com</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Codeforces 986E - Prince's Problem (Tree, DS, Math)</t>
+          <t>ICPC Team Notebook - 25 Trang</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>2800</t>
+          <t>Teamwork</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Re-solve bài cũ</t>
+          <t>Checklist</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
@@ -1405,37 +1405,37 @@
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-11-06 (Thứ Sáu)</t>
+          <t>2026-11-04 (Thứ Tư)</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Tuần 3: Cấu trúc dữ liệu nâng cao &amp; Chia căn (Mo, Sqrt Decomposition, SegTree)</t>
+          <t>Tuần 3: TỔNG LỰC CHUẨN BỊ CHO KỲ THI ICPC QUỐC GIA 2026</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Ladder 16: Data Structures &amp; Hashing</t>
+          <t>Rà soát bẫy tràn số (MOD, 64-bit, fast I/O) &amp; Viết test generator</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/problemset/problem/126/B</t>
+          <t>https://codeforces.com/contest/786/problem/B</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Codeforces 126B - Password</t>
+          <t>Codeforces 786B - Segment Tree trên đồ thị</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>1700</t>
+          <t>2200</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Ladder 16 Re-solve</t>
+          <t>Stress Test Lab</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
@@ -1447,37 +1447,37 @@
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-11-07 (Thứ Bảy)</t>
+          <t>2026-11-05 (Thứ Năm)</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Tuần 3: Cấu trúc dữ liệu nâng cao &amp; Chia căn (Mo, Sqrt Decomposition, SegTree)</t>
+          <t>Tuần 3: TỔNG LỰC CHUẨN BỊ CHO KỲ THI ICPC QUỐC GIA 2026</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Review Template SegTree Lazy &amp; Fenwick 2D</t>
+          <t>Chiến thuật tâm lý thi đấu 3 người 1 máy vòng Quốc Gia</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>https://oj.vnoi.info/problem/segtree_itteq1</t>
+          <t>https://codeforces.com</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>VNOI ITTEQ1 - Segment Tree nâng cao</t>
+          <t>Họp chiến thuật Team ICPC</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Strategy</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Review Template</t>
+          <t>Team Meeting</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
@@ -1487,81 +1487,81 @@
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>2026-11-08 (Chủ Nhật)</t>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-06 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Tuần 3: Cấu trúc dữ liệu nâng cao &amp; Chia căn (Mo, Sqrt Decomposition, SegTree)</t>
+          <t>Tuần 3: TỔNG LỰC CHUẨN BỊ CHO KỲ THI ICPC QUỐC GIA 2026</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>MOCK TEST 3: ICPC Regional Simulation 5 Giờ (Team Contest #3)</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>https://codeforces.com/gym/103449</t>
-        </is>
-      </c>
-      <c r="E22" s="10" t="inlineStr">
-        <is>
-          <t>2021-2022 ICPC Asia Hanoi Regional Contest</t>
+          <t>Thư giãn, ngủ đủ giấc, chuẩn bị tài khoản và máy thi</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>https://codeforces.com</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Nghỉ ngơi nạp năng lượng trước Vòng Quốc Gia</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>ICPC Team</t>
-        </is>
-      </c>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>FULL MOCK TEST</t>
-        </is>
-      </c>
-      <c r="H22" s="11" t="inlineStr">
-        <is>
-          <t>Chưa làm</t>
+          <t>Rest</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Rest &amp; Recharge</t>
+        </is>
+      </c>
+      <c r="H22" s="12" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2026-11-09 (Thứ Hai)</t>
+          <t>2026-11-07 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Tuần 4: Toán học, Tổ hợp, Nghịch đảo Modulo &amp; Hình học Sweepline</t>
+          <t>Tuần 4: KỲ THI ICPC QUỐC GIA 2026 (08-09/11) &amp; BƯỚC NGOẶT CHUYỂN GIAO</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Bao hàm loại trừ &amp; Lucas Theorem: Re-solve bài cũ</t>
+          <t>Thử máy Kỳ thi ICPC Quốc gia 2026 tại điểm thi tập trung</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/contest/1043/problem/F</t>
+          <t>https://codeforces.com/gyms</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Codeforces 1043F - Make It One (Bao hàm)</t>
+          <t>ICPC Vietnam National 2026 - Practice Session</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>2400</t>
+          <t>ICPC Team</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Re-solve bài cũ</t>
+          <t>THỬ MÁY</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
@@ -1573,37 +1573,37 @@
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-11-10 (Thứ Ba)</t>
+          <t>2026-11-08 (Chủ Nhật)</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Tuần 4: Toán học, Tổ hợp, Nghịch đảo Modulo &amp; Hình học Sweepline</t>
+          <t>Tuần 4: KỲ THI ICPC QUỐC GIA 2026 (08-09/11) &amp; BƯỚC NGOẶT CHUYỂN GIAO</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Toán chia kẹo Euler &amp; Nghịch đảo modulo</t>
+          <t>CHÍNH THỨC THI ICPC QUỐC GIA 2026 (VIETNAM NATIONAL - 5 GIỜ)</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>https://oj.vnoi.info/problem/c11tct</t>
+          <t>https://codeforces.com/gyms</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>VNOI c11tct - Chia kẹo, Lucas theory</t>
+          <t>2026 ICPC Vietnam National Contest</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>ICPC Team</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>VNOI Math</t>
+          <t>OFFICIAL CONTEST</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
@@ -1615,37 +1615,37 @@
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-11-11 (Thứ Tư)</t>
+          <t>2026-11-09 (Thứ Hai)</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Tuần 4: Toán học, Tổ hợp, Nghịch đảo Modulo &amp; Hình học Sweepline</t>
+          <t>Tuần 4: KỲ THI ICPC QUỐC GIA 2026 (08-09/11) &amp; BƯỚC NGOẶT CHUYỂN GIAO</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Kiểm tra cá nhân OLP Mock Contest #4 (3h - Toán &amp; Tổ hợp)</t>
+          <t>Tổng kết kết quả vòng Quốc gia &amp; Xác định slot dự Regional Đà Nẵng</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/contest/1974</t>
+          <t>https://olp.vn</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Codeforces Round 946</t>
+          <t>Bảng điểm ICPC Quốc Gia 2026</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Div.3/2</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>OLP Mock Test</t>
+          <t>Debrief</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
@@ -1657,32 +1657,32 @@
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-11-12 (Thứ Năm)</t>
+          <t>2026-11-10 (Thứ Ba)</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Tuần 4: Toán học, Tổ hợp, Nghịch đảo Modulo &amp; Hình học Sweepline</t>
+          <t>Tuần 4: KỲ THI ICPC QUỐC GIA 2026 (08-09/11) &amp; BƯỚC NGOẶT CHUYỂN GIAO</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Hình học Sweepline &amp; Convex Hull: Re-solve bài cũ</t>
+          <t>Upsolving toàn bộ các bài trong tầm với đề ICPC Quốc Gia 2026</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/contest/529/problem/C</t>
+          <t>https://codeforces.com/contest/1043/problem/F</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Codeforces 529C - Sweepline (Rooks Defender)</t>
+          <t>Codeforces 1043F - Make It One (Bao hàm loại trừ)</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>2400</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
@@ -1699,27 +1699,27 @@
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2026-11-13 (Thứ Sáu)</t>
+          <t>2026-11-11 (Thứ Tư)</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Tuần 4: Toán học, Tổ hợp, Nghịch đảo Modulo &amp; Hình học Sweepline</t>
+          <t>Tuần 4: KỲ THI ICPC QUỐC GIA 2026 (08-09/11) &amp; BƯỚC NGOẶT CHUYỂN GIAO</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Hình học tính toán &amp; Bao lồi (Monotone Chain)</t>
+          <t>Khởi động giai đoạn 2: Ôn luyện cá nhân Olympic Tin học SV</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>https://oj.vnoi.info/problem/cavli</t>
+          <t>https://oj.vnoi.info/problem/c11tct</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>VNOI cavli - Hình học, Bao lồi</t>
+          <t>VNOI c11tct - Chia kẹo Euler &amp; Lucas</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Geometry</t>
+          <t>OLP Practice</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
@@ -1741,82 +1741,82 @@
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-11-14 (Thứ Bảy)</t>
+          <t>2026-11-12 (Thứ Năm)</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Tuần 4: Toán học, Tổ hợp, Nghịch đảo Modulo &amp; Hình học Sweepline</t>
+          <t>Tuần 4: KỲ THI ICPC QUỐC GIA 2026 (08-09/11) &amp; BƯỚC NGOẶT CHUYỂN GIAO</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
+          <t>Toán học &amp; Tổ hợp: Re-solve các bài toán chia kẹo, nghịch đảo</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>https://oj.vnoi.info/problem/fc090_divcan</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>VNOI fc090_divcan - Bao hàm, Lucas</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>Re-solve</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-13 (Thứ Sáu)</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Tuần 4: KỲ THI ICPC QUỐC GIA 2026 (08-09/11) &amp; BƯỚC NGOẶT CHUYỂN GIAO</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
           <t>Ladder 16: Math &amp; Number Theory</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>https://codeforces.com/problemset/problem/354/C</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>Codeforces 354C - Vasya and Beautiful Arrays</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>2100</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="G29" s="6" t="inlineStr">
         <is>
           <t>Ladder 16 Re-solve</t>
         </is>
       </c>
-      <c r="H28" s="7" t="inlineStr">
-        <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t>2026-11-15 (Chủ Nhật)</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Tuần 4: Toán học, Tổ hợp, Nghịch đảo Modulo &amp; Hình học Sweepline</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>MOCK TEST 4: ICPC Regional Simulation 5 Giờ (Team Contest #4)</t>
-        </is>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
-        <is>
-          <t>https://codeforces.com/gym/104639</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="inlineStr">
-        <is>
-          <t>2023-2024 ICPC Asia Hue Regional Contest</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>ICPC Team</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>FULL MOCK TEST</t>
-        </is>
-      </c>
-      <c r="H29" s="11" t="inlineStr">
+      <c r="H29" s="7" t="inlineStr">
         <is>
           <t>Chưa làm</t>
         </is>
@@ -1825,37 +1825,37 @@
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-11-16 (Thứ Hai)</t>
+          <t>2026-11-14 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Tuần 5: Thuật toán Xâu ký tự (Strings), Luồng cực đại (Flow) &amp; Game Theory</t>
+          <t>Tuần 5: Chuyên sâu Olympic: Hình học Sweepline, Bao lồi &amp; CTDL Nâng cao</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>KMP, Z-function &amp; Hash 2D: Re-solve bài cũ</t>
+          <t>Hình học tính toán: Bao lồi (Monotone Chain / Graham Scan)</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/problemset/problem/432/D</t>
+          <t>https://oj.vnoi.info/problem/cavli</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Codeforces 432D - Prefixes and Suffixes</t>
+          <t>VNOI cavli - Hình học, Bao lồi</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>Ladder 16 Re-solve</t>
+          <t>Geometry</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
@@ -1867,37 +1867,37 @@
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-11-17 (Thứ Ba)</t>
+          <t>2026-11-15 (Chủ Nhật)</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Tuần 5: Thuật toán Xâu ký tự (Strings), Luồng cực đại (Flow) &amp; Game Theory</t>
+          <t>Tuần 5: Chuyên sâu Olympic: Hình học Sweepline, Bao lồi &amp; CTDL Nâng cao</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Aho-Corasick &amp; DP trên Trie</t>
+          <t>MOCK TEST OLP #1: Đề thi Siêu Cúp / Chuyên Tin các năm (3.5 giờ)</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>https://lqdoj.edu.vn/problem/lqdoj2022r4ugpalind</t>
+          <t>https://cms.ioi-jp.org/joi2023-sp1-open</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>LQDOJ ugpalind - DP + Aho-Corasick</t>
+          <t>JOI Spring Camp 2023 Contest 1</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>JOI</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>LQDOJ String</t>
+          <t>OLP Mock Test</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
@@ -1909,37 +1909,37 @@
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-11-18 (Thứ Tư)</t>
+          <t>2026-11-16 (Thứ Hai)</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Tuần 5: Thuật toán Xâu ký tự (Strings), Luồng cực đại (Flow) &amp; Game Theory</t>
+          <t>Tuần 5: Chuyên sâu Olympic: Hình học Sweepline, Bao lồi &amp; CTDL Nâng cao</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Kiểm tra cá nhân OLP Mock Contest #5 (3.5h - Đề Siêu Cúp / Chuyên Tin)</t>
+          <t>Sweepline quét tọa độ X kết hợp Segment Tree</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>https://cms.ioi-jp.org/joi2023-sp1-open</t>
+          <t>https://codeforces.com/contest/529/problem/C</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>JOI Spring Camp 2023 Contest 1</t>
+          <t>Codeforces 529C - Sweepline (Rooks Defender)</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>JOI</t>
+          <t>2200</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>OLP Mock Test</t>
+          <t>Re-solve bài cũ</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
@@ -1951,32 +1951,32 @@
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-11-19 (Thứ Năm)</t>
+          <t>2026-11-17 (Thứ Ba)</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Tuần 5: Thuật toán Xâu ký tự (Strings), Luồng cực đại (Flow) &amp; Game Theory</t>
+          <t>Tuần 5: Chuyên sâu Olympic: Hình học Sweepline, Bao lồi &amp; CTDL Nâng cao</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Luồng cực đại (Dinic) &amp; Cặp ghép cực đại</t>
+          <t>Persistent Segment Tree &amp; Treap: Re-solve bài cũ</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/contest/944/problem/F</t>
+          <t>https://codeforces.com/contest/986/problem/E</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Codeforces 944F - CTDL, Game</t>
+          <t>Codeforces 986E - Prince's Problem (Tree, DS, Math)</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>2400</t>
+          <t>2800</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
@@ -1993,37 +1993,37 @@
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-11-20 (Thứ Sáu)</t>
+          <t>2026-11-18 (Thứ Tư)</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Tuần 5: Thuật toán Xâu ký tự (Strings), Luồng cực đại (Flow) &amp; Game Theory</t>
+          <t>Tuần 5: Chuyên sâu Olympic: Hình học Sweepline, Bao lồi &amp; CTDL Nâng cao</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Game Theory: Nim, Sprague-Grundy &amp; Nhận xét Adhoc</t>
+          <t>Kỹ thuật Chia căn lớn bé &amp; DSU</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/contest/2181/problem/F</t>
+          <t>https://oj.vnoi.info/problem/coci1920_o_paint</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Codeforces 2181F - Fragmented Nim</t>
+          <t>COCI 1920 Paint - Chia căn lớn bé &amp; DSU</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>1600</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>Re-solve bài cũ</t>
+          <t>Data Structures</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
@@ -2035,17 +2035,17 @@
     <row r="35" ht="22" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-11-21 (Thứ Bảy)</t>
+          <t>2026-11-19 (Thứ Năm)</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Tuần 5: Thuật toán Xâu ký tự (Strings), Luồng cực đại (Flow) &amp; Game Theory</t>
+          <t>Tuần 5: Chuyên sâu Olympic: Hình học Sweepline, Bao lồi &amp; CTDL Nâng cao</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Ladder 16: KMP String Differencing</t>
+          <t>Ladder 16: KMP Differencing</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -2077,37 +2077,37 @@
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-11-22 (Chủ Nhật)</t>
+          <t>2026-11-20 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Tuần 5: Thuật toán Xâu ký tự (Strings), Luồng cực đại (Flow) &amp; Game Theory</t>
+          <t>Tuần 5: Chuyên sâu Olympic: Hình học Sweepline, Bao lồi &amp; CTDL Nâng cao</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>MOCK TEST 5: ICPC Vietnam National Simulation 5 Giờ (Team Contest #5)</t>
+          <t>Review Template SegTree Lazy &amp; Fenwick 2D</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/gym/104725</t>
+          <t>https://oj.vnoi.info/problem/segtree_itteq1</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>2023 ICPC Vietnam National Contest</t>
+          <t>VNOI ITTEQ1 - Segment Tree nâng cao</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>ICPC Team</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>FULL MOCK TEST</t>
+          <t>Review Template</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
@@ -2119,37 +2119,37 @@
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-11-23 (Thứ Hai)</t>
+          <t>2026-11-21 (Thứ Bảy)</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Tuần 6: Tổng lực Luyện đề, Chiến thuật Team &amp; Stress Testing</t>
+          <t>Tuần 6: Xâu ký tự (Strings), Luồng cực đại (Flow) &amp; Game Theory</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Upsolving bài khó Mock Test 5 &amp; Phân tích bug phòng thi</t>
+          <t>KMP, Z-function &amp; Hash 2D: Re-solve bài cũ</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/contest/1442/problem/C</t>
+          <t>https://codeforces.com/problemset/problem/432/D</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Codeforces 1442C - Graph, Shortest Path</t>
+          <t>Codeforces 432D - Prefixes and Suffixes</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>2400</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>Re-solve bài cũ</t>
+          <t>Ladder 16 Re-solve</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
@@ -2159,42 +2159,42 @@
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-24 (Thứ Ba)</t>
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>2026-11-22 (Chủ Nhật)</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Tuần 6: Tổng lực Luyện đề, Chiến thuật Team &amp; Stress Testing</t>
+          <t>Tuần 6: Xâu ký tự (Strings), Luồng cực đại (Flow) &amp; Game Theory</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Re-solve bài cũ: DSU on Tree / Small to large</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>https://codeforces.com/problemset/problem/570/D</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>Codeforces 570D - Tree Requests</t>
+          <t>MOCK TEST REGIONAL #4: 2023-2024 ICPC Asia Hue Regional Contest (5h)</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/gym/104639</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
+        <is>
+          <t>2023-2024 ICPC Asia Hue Regional Contest</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>2200</t>
-        </is>
-      </c>
-      <c r="G38" s="6" t="inlineStr">
-        <is>
-          <t>Ladder 16 Re-solve</t>
-        </is>
-      </c>
-      <c r="H38" s="7" t="inlineStr">
+          <t>ICPC Team</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>FULL MOCK TEST</t>
+        </is>
+      </c>
+      <c r="H38" s="11" t="inlineStr">
         <is>
           <t>Chưa làm</t>
         </is>
@@ -2203,37 +2203,37 @@
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2026-11-25 (Thứ Tư)</t>
+          <t>2026-11-23 (Thứ Hai)</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Tuần 6: Tổng lực Luyện đề, Chiến thuật Team &amp; Stress Testing</t>
+          <t>Tuần 6: Xâu ký tự (Strings), Luồng cực đại (Flow) &amp; Game Theory</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Kiểm tra cá nhân OLP Mock Contest #6 (3h - Đề Olympic các năm)</t>
+          <t>Aho-Corasick &amp; DP trên Trie</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>https://oj.vnoi.info/problem/voi21_rmat</t>
+          <t>https://lqdoj.edu.vn/problem/lqdoj2022r4ugpalind</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>VOI 2021 RMAT - Observation &amp; Matrix</t>
+          <t>LQDOJ ugpalind - DP + Aho-Corasick</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>VOI</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>OLP Mock Test</t>
+          <t>LQDOJ String</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
@@ -2245,27 +2245,27 @@
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-11-26 (Thứ Năm)</t>
+          <t>2026-11-24 (Thứ Ba)</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Tuần 6: Tổng lực Luyện đề, Chiến thuật Team &amp; Stress Testing</t>
+          <t>Tuần 6: Xâu ký tự (Strings), Luồng cực đại (Flow) &amp; Game Theory</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Kiểm tra và hoàn thiện ICPC Team Notebook (Codeforces Template)</t>
+          <t>Luồng cực đại (Dinic) &amp; Cặp ghép hai phía</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/contest/1697/problem/E</t>
+          <t>https://codeforces.com/contest/944/problem/F</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Codeforces 1697E - Graph, DP, Tổ hợp</t>
+          <t>Codeforces 944F - CTDL, Game</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
@@ -2287,37 +2287,37 @@
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2026-11-27 (Thứ Sáu)</t>
+          <t>2026-11-25 (Thứ Tư)</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Tuần 6: Tổng lực Luyện đề, Chiến thuật Team &amp; Stress Testing</t>
+          <t>Tuần 6: Xâu ký tự (Strings), Luồng cực đại (Flow) &amp; Game Theory</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Thực hành Stress Test (Viết script sinh test ngẫu nhiên đối chiếu)</t>
+          <t>Game Theory: Nim, Sprague-Grundy &amp; Nhận xét Adhoc</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>https://dmoj.ca/problem/coci06c1p6</t>
+          <t>https://codeforces.com/contest/2181/problem/F</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>COCI 06 c1p6 - Hash 2D</t>
+          <t>Codeforces 2181F - Fragmented Nim</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>1600</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>Stress Test Lab</t>
+          <t>Re-solve bài cũ</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
@@ -2329,27 +2329,27 @@
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-11-28 (Thứ Bảy)</t>
+          <t>2026-11-26 (Thứ Năm)</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Tuần 6: Tổng lực Luyện đề, Chiến thuật Team &amp; Stress Testing</t>
+          <t>Tuần 6: Xâu ký tự (Strings), Luồng cực đại (Flow) &amp; Game Theory</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Review toàn bộ các Trick lỏ &amp; bẫy tràn số (Overflow, MOD, 1LL&lt;&lt;x)</t>
+          <t>DSU on tree (Small to large) kết hợp Bitmask</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/contest/786/problem/B</t>
+          <t>https://codeforces.com/problemset/problem/570/D</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Codeforces 786B - Dijkstra đoạn</t>
+          <t>Codeforces 570D - Tree Requests</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>Trick lỏ</t>
+          <t>Ladder 16 Re-solve</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
@@ -2371,82 +2371,82 @@
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2026-11-29 (Chủ Nhật)</t>
+          <t>2026-11-27 (Thứ Sáu)</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Tuần 6: Tổng lực Luyện đề, Chiến thuật Team &amp; Stress Testing</t>
+          <t>Tuần 6: Xâu ký tự (Strings), Luồng cực đại (Flow) &amp; Game Theory</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>MOCK TEST 6: FINAL FULL ICPC SIMULATION 5 GIỜ</t>
+          <t>Kiểm tra tiến độ 137 bài khó đã re-solve được bao nhiêu bài</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/gym/103960</t>
+          <t>https://codeforces.com/contest/1442/problem/C</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>2022-2023 ICPC Brazil Subregional / Asia Archive</t>
+          <t>Codeforces 1442C - Graph, Shortest Path</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
+          <t>2400</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>Re-solve bài cũ</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>2026-11-28 (Thứ Bảy)</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Tuần 7: Tổng duyệt cuối cùng &amp; Chuẩn bị lên đường đi Đà Nẵng</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>FINAL MOCK TEST: 2022-2023 ICPC Asia Yokohama Regional (5 Giờ)</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/gym/104021</t>
+        </is>
+      </c>
+      <c r="E44" s="10" t="inlineStr">
+        <is>
+          <t>2022-2023 ICPC Asia Yokohama Regional</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
           <t>ICPC Team</t>
         </is>
       </c>
-      <c r="G43" s="6" t="inlineStr">
+      <c r="G44" s="8" t="inlineStr">
         <is>
           <t>FINAL MOCK TEST</t>
         </is>
       </c>
-      <c r="H43" s="7" t="inlineStr">
-        <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-30 (Thứ Hai)</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>Tuần 7: Tapering, Thư giãn trí não &amp; Rà soát lần cuối trước giờ G</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>Re-solve nhẹ nhàng: Ladder 16 các bài trung bình (Lấy cảm giác tay)</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>https://codeforces.com/problemset/problem/476/B</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr">
-        <is>
-          <t>Codeforces 476B - Dreamoon and WiFi</t>
-        </is>
-      </c>
-      <c r="F44" s="5" t="inlineStr">
-        <is>
-          <t>1300</t>
-        </is>
-      </c>
-      <c r="G44" s="6" t="inlineStr">
-        <is>
-          <t>Ladder 16</t>
-        </is>
-      </c>
-      <c r="H44" s="7" t="inlineStr">
+      <c r="H44" s="11" t="inlineStr">
         <is>
           <t>Chưa làm</t>
         </is>
@@ -2455,37 +2455,37 @@
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026-12-01 (Thứ Ba)</t>
+          <t>2026-11-29 (Chủ Nhật)</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Tuần 7: Tapering, Thư giãn trí não &amp; Rà soát lần cuối trước giờ G</t>
+          <t>Tuần 7: Tổng duyệt cuối cùng &amp; Chuẩn bị lên đường đi Đà Nẵng</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Rà soát lại danh sách 137 bài khó đã ôn tập</t>
+          <t>MOCK TEST OLP #2: Đề Olympic Tin học Sinh viên Toàn quốc (3.5 Giờ)</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com/contest/2181/problem/D</t>
+          <t>https://oj.vnoi.info/problem/voi21_rmat</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Codeforces 2181D - Doorway (BS + DS)</t>
+          <t>VOI 2021 RMAT - Observation &amp; Matrix</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>VOI</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>Re-solve nhẹ</t>
+          <t>OLP Mock Test</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
@@ -2497,37 +2497,37 @@
     <row r="46" ht="22" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-12-02 (Thứ Tư)</t>
+          <t>2026-11-30 (Thứ Hai)</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Tuần 7: Tapering, Thư giãn trí não &amp; Rà soát lần cuối trước giờ G</t>
+          <t>Tuần 7: Tổng duyệt cuối cùng &amp; Chuẩn bị lên đường đi Đà Nẵng</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Kiểm tra Template Notebook, máy chấm, compiler flags (-O2, -fsanitize)</t>
+          <t>Upsolve bài khó Mock Test &amp; Đóng gói toàn bộ code mẫu</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>https://codeforces.com</t>
+          <t>https://codeforces.com/contest/1697/problem/E</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Chuẩn bị môi trường thi &amp; template in ấn</t>
+          <t>Codeforces 1697E - Graph, DP, Tổ hợp</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Preparation</t>
+          <t>2400</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>Checklist</t>
+          <t>Re-solve bài cũ</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
@@ -2539,17 +2539,17 @@
     <row r="47" ht="22" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2026-12-03 (Thứ Năm)</t>
+          <t>2026-12-01 (Thứ Ba)</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Tuần 7: Tapering, Thư giãn trí não &amp; Rà soát lần cuối trước giờ G</t>
+          <t>Tuần 7: Tổng duyệt cuối cùng &amp; Chuẩn bị lên đường đi Đà Nẵng</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Chiến thuật tâm lý: Phân bổ thời gian, nhận diện bài bẫy</t>
+          <t>In ấn Team Notebook bản cứng (25 trang chuẩn ICPC quốc tế)</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -2559,17 +2559,17 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Họp chiến thuật team ICPC</t>
+          <t>In ấn Team Notebook</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Strategy</t>
+          <t>Preparation</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>Team Meeting</t>
+          <t>Checklist</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
@@ -2581,17 +2581,17 @@
     <row r="48" ht="22" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-12-04 (Thứ Sáu)</t>
+          <t>2026-12-02 (Thứ Tư)</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Tuần 7: Tapering, Thư giãn trí não &amp; Rà soát lần cuối trước giờ G</t>
+          <t>Tuần 7: Tổng duyệt cuối cùng &amp; Chuẩn bị lên đường đi Đà Nẵng</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Nghỉ ngơi, ngủ đủ giấc, chuẩn bị thẻ sinh viên &amp; CCCD</t>
+          <t>Kiểm tra compiler flags (-O2, -fsanitize=undefined) &amp; máy chấm</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -2601,104 +2601,398 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Nghỉ ngơi chuẩn bị cho ngày thi</t>
+          <t>Kiểm tra môi trường thi</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Rest</t>
+          <t>Preparation</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>Rest &amp; Recharge</t>
-        </is>
-      </c>
-      <c r="H48" s="12" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
+          <t>Checklist</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
         </is>
       </c>
     </row>
     <row r="49" ht="22" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
+          <t>2026-12-03 (Thứ Năm)</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Tuần 7: Tổng duyệt cuối cùng &amp; Chuẩn bị lên đường đi Đà Nẵng</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Họp chiến thuật team 3 người 1 máy lần cuối trước khi bay</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>https://codeforces.com</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Họp chiến thuật Team ICPC</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>Team Meeting</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-04 (Thứ Sáu)</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Tuần 7: Tổng duyệt cuối cùng &amp; Chuẩn bị lên đường đi Đà Nẵng</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Nghỉ ngơi, chuẩn bị hành lý, giấy tờ tùy thân và vé đi Đà Nẵng</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>https://codeforces.com</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Nghỉ ngơi và chuẩn bị lên đường</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Rest</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>Rest &amp; Recharge</t>
+        </is>
+      </c>
+      <c r="H50" s="12" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
           <t>2026-12-05 (Thứ Bảy)</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>Tuần 7: Tapering, Thư giãn trí não &amp; Rà soát lần cuối trước giờ G</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t>NGÀY THI OLYMPIC TIN HỌC SINH VIÊN (CÁ NHÂN)</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Tuần 8: VÒNG CHUNG KẾT TOÀN QUỐC OLP'26 &amp; ICPC ASIA DANANG 2026 (TẠI VKU)</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Di chuyển đến TP. Đà Nẵng, nhận phòng &amp; ổn định nơi lưu trú</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
         <is>
           <t>https://olp.vn</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>Olympic Tin học Sinh viên Toàn quốc</t>
-        </is>
-      </c>
-      <c r="F49" s="5" t="inlineStr">
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Có mặt tại Đà Nẵng</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>Check-in</t>
+        </is>
+      </c>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-06 (Chủ Nhật)</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Tuần 8: VÒNG CHUNG KẾT TOÀN QUỐC OLP'26 &amp; ICPC ASIA DANANG 2026 (TẠI VKU)</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Tham quan Trường ĐH CNTT và Truyền thông Việt - Hàn (VKU Đà Nẵng)</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>https://olp.vn</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Thăm quan địa điểm thi VKU Đà Nẵng</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>Site Visit</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>Venue Tour</t>
+        </is>
+      </c>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-07 (Thứ Hai)</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Tuần 8: VÒNG CHUNG KẾT TOÀN QUỐC OLP'26 &amp; ICPC ASIA DANANG 2026 (TẠI VKU)</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Gõ code nhẹ nhàng vài bài cơ bản lấy cảm giác phím mượt mà</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>https://codeforces.com/problemset/problem/476/B</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Codeforces 476B - Dreamoon and WiFi</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>1300</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>Warm-up</t>
+        </is>
+      </c>
+      <c r="H53" s="7" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-08 (Thứ Ba)</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Tuần 8: VÒNG CHUNG KẾT TOÀN QUỐC OLP'26 &amp; ICPC ASIA DANANG 2026 (TẠI VKU)</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>ĐĂNG KÝ THAM GIA OLP &amp; ICPC ASIA DANANG TẠI VKU; CHUNG KẾT OLYMPIC AI</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>https://olp.vn</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Đăng ký OLP'26 &amp; ICPC Asia Danang (08/12/2026)</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Registration</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>OFFICIAL EVENT</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-09 (Thứ Tư)</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Tuần 8: VÒNG CHUNG KẾT TOÀN QUỐC OLP'26 &amp; ICPC ASIA DANANG 2026 (TẠI VKU)</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>CHÍNH THỨC THI OLYMPIC TIN HỌC SINH VIÊN (OLP'26) - KHỐI CHUYÊN TIN &amp; SIÊU CÚP</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>https://olp.vn</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Kỳ thi Cá nhân Olympic Tin học SV 2026 (09/12/2026)</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
         <is>
           <t>CONTEST</t>
         </is>
       </c>
-      <c r="G49" s="6" t="inlineStr">
+      <c r="G55" s="6" t="inlineStr">
         <is>
           <t>OFFICIAL CONTEST</t>
         </is>
       </c>
-      <c r="H49" s="7" t="inlineStr">
+      <c r="H55" s="7" t="inlineStr">
         <is>
           <t>Đến giờ G!</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="8" t="inlineStr">
-        <is>
-          <t>2026-12-06 (Chủ Nhật)</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>Tuần 7: Tapering, Thư giãn trí não &amp; Rà soát lần cuối trước giờ G</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>NGÀY THI ICPC REGIONAL (TEAM 3 NGƯỜI / 5 GIỜ)</t>
-        </is>
-      </c>
-      <c r="D50" s="9" t="inlineStr">
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-10 (Thứ Năm)</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Tuần 8: VÒNG CHUNG KẾT TOÀN QUỐC OLP'26 &amp; ICPC ASIA DANANG 2026 (TẠI VKU)</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>KHAI MẠC ICPC ASIA DANANG 2026; THỬ MÁY (PRACTICE SESSION 2H) &amp; NỘP NOTEBOOK</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>https://olp.vn</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Khai mạc &amp; Thử máy ICPC Asia Danang (10/12/2026)</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>Practice</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>OFFICIAL EVENT</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>Đến giờ G!</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-11 (Thứ Sáu)</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Tuần 8: VÒNG CHUNG KẾT TOÀN QUỐC OLP'26 &amp; ICPC ASIA DANANG 2026 (TẠI VKU)</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>CHÍNH THỨC THI LẬP TRÌNH QUỐC TẾ ICPC ASIA DANANG 2026 (5 TIẾNG: 08:00 - 13:00)</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
         <is>
           <t>https://icpc.global</t>
         </is>
       </c>
-      <c r="E50" s="10" t="inlineStr">
-        <is>
-          <t>ICPC Asia Regional Contest</t>
-        </is>
-      </c>
-      <c r="F50" s="5" t="inlineStr">
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Chính thức thi ICPC Asia Danang 2026 (11/12/2026)</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
         <is>
           <t>CONTEST</t>
         </is>
       </c>
-      <c r="G50" s="8" t="inlineStr">
+      <c r="G57" s="6" t="inlineStr">
         <is>
           <t>OFFICIAL CONTEST</t>
         </is>
       </c>
-      <c r="H50" s="11" t="inlineStr">
+      <c r="H57" s="7" t="inlineStr">
         <is>
           <t>Đến giờ G!</t>
         </is>
@@ -5114,12 +5408,12 @@
       <c r="C93" s="5" t="inlineStr"/>
       <c r="D93" s="16" t="inlineStr">
         <is>
-          <t>https://codeforces.com/problemset/problem/1991/E</t>
+          <t>https://codeforces.com/problemset/problem/1991/D</t>
         </is>
       </c>
       <c r="E93" s="17" t="inlineStr">
         <is>
-          <t>constructive algorithms, dfs and similar, games (Ôn lại: 809 ngày)</t>
+          <t>bitmasks, constructive algorithms, graphs (Ôn lại: 809 ngày)</t>
         </is>
       </c>
       <c r="F93" s="5" t="inlineStr">
@@ -5138,12 +5432,12 @@
       <c r="C94" s="5" t="inlineStr"/>
       <c r="D94" s="16" t="inlineStr">
         <is>
-          <t>https://codeforces.com/problemset/problem/1991/D</t>
+          <t>https://codeforces.com/problemset/problem/1991/E</t>
         </is>
       </c>
       <c r="E94" s="17" t="inlineStr">
         <is>
-          <t>bitmasks, constructive algorithms, graphs (Ôn lại: 809 ngày)</t>
+          <t>constructive algorithms, dfs and similar, games (Ôn lại: 808 ngày)</t>
         </is>
       </c>
       <c r="F94" s="5" t="inlineStr">
@@ -5167,7 +5461,7 @@
       </c>
       <c r="E95" s="17" t="inlineStr">
         <is>
-          <t>brute force, dfs and similar, graphs (Ôn lại: 358 ngày)</t>
+          <t>brute force, dfs and similar, graphs (Ôn lại: 357 ngày)</t>
         </is>
       </c>
       <c r="F95" s="5" t="inlineStr">
@@ -5311,7 +5605,7 @@
       </c>
       <c r="E101" s="17" t="inlineStr">
         <is>
-          <t>graphs, greedy, math (Ôn lại: 332 ngày)</t>
+          <t>graphs, greedy, math (Ôn lại: 331 ngày)</t>
         </is>
       </c>
       <c r="F101" s="5" t="inlineStr">
@@ -5952,7 +6246,7 @@
       </c>
       <c r="B136" s="17" t="inlineStr">
         <is>
-          <t>dfs and similar, graphs, trees (Ôn lại: 844 ngày)</t>
+          <t>dfs and similar, graphs, trees (Ôn lại: 843 ngày)</t>
         </is>
       </c>
       <c r="C136" s="5" t="inlineStr">
@@ -7235,7 +7529,7 @@
       </c>
       <c r="E44" s="17" t="inlineStr">
         <is>
-          <t>binary search, data structures, greedy (Ôn lại: 330 ngày)</t>
+          <t>binary search, data structures, greedy (Ôn lại: 329 ngày)</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
@@ -7318,12 +7612,12 @@
       <c r="C47" s="5" t="inlineStr"/>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>https://codeforces.com/problemset/problem/1991/E</t>
+          <t>https://codeforces.com/problemset/problem/1991/D</t>
         </is>
       </c>
       <c r="E47" s="17" t="inlineStr">
         <is>
-          <t>constructive algorithms, dfs and similar, games (Ôn lại: 809 ngày)</t>
+          <t>bitmasks, constructive algorithms, graphs (Ôn lại: 809 ngày)</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
@@ -7350,12 +7644,12 @@
       </c>
       <c r="D48" s="16" t="inlineStr">
         <is>
-          <t>https://codeforces.com/problemset/problem/1991/D</t>
+          <t>https://codeforces.com/problemset/problem/1991/E</t>
         </is>
       </c>
       <c r="E48" s="17" t="inlineStr">
         <is>
-          <t>bitmasks, constructive algorithms, graphs (Ôn lại: 809 ngày)</t>
+          <t>constructive algorithms, dfs and similar, games (Ôn lại: 808 ngày)</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
@@ -7615,7 +7909,7 @@
       </c>
       <c r="E57" s="17" t="inlineStr">
         <is>
-          <t>greedy, math, number theory (Ôn lại: 844 ngày)</t>
+          <t>greedy, math, number theory (Ôn lại: 843 ngày)</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
@@ -7703,7 +7997,7 @@
       </c>
       <c r="E60" s="17" t="inlineStr">
         <is>
-          <t>greedy, math (Ôn lại: 357 ngày)</t>
+          <t>greedy, math (Ôn lại: 356 ngày)</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
@@ -7791,7 +8085,7 @@
       </c>
       <c r="E63" s="17" t="inlineStr">
         <is>
-          <t>graphs, greedy, math (Ôn lại: 332 ngày)</t>
+          <t>graphs, greedy, math (Ôn lại: 331 ngày)</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
@@ -8328,7 +8622,7 @@
       </c>
       <c r="B92" s="17" t="inlineStr">
         <is>
-          <t>combinatorics, dp, math (Ôn lại: 330 ngày)</t>
+          <t>combinatorics, dp, math (Ôn lại: 329 ngày)</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
@@ -8428,7 +8722,7 @@
       </c>
       <c r="B97" s="17" t="inlineStr">
         <is>
-          <t>dp, sortings, string suffix structures (Ôn lại: 358 ngày)</t>
+          <t>dp, sortings, string suffix structures (Ôn lại: 357 ngày)</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
@@ -8788,7 +9082,7 @@
       </c>
       <c r="B115" s="17" t="inlineStr">
         <is>
-          <t>constructive algorithms, dp (Ôn lại: 357 ngày)</t>
+          <t>constructive algorithms, dp (Ôn lại: 356 ngày)</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
@@ -10095,7 +10389,7 @@
       </c>
       <c r="E38" s="17" t="inlineStr">
         <is>
-          <t>data structures, sortings (Ôn lại: 357 ngày)</t>
+          <t>data structures, sortings (Ôn lại: 356 ngày)</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
@@ -10283,7 +10577,7 @@
       </c>
       <c r="E44" s="17" t="inlineStr">
         <is>
-          <t>binary search, data structures, greedy (Ôn lại: 330 ngày)</t>
+          <t>binary search, data structures, greedy (Ôn lại: 329 ngày)</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
@@ -12031,7 +12325,7 @@
       </c>
       <c r="E43" s="17" t="inlineStr">
         <is>
-          <t>geometry (Ôn lại: 332 ngày)</t>
+          <t>geometry (Ôn lại: 331 ngày)</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
@@ -12408,7 +12702,7 @@
       </c>
       <c r="B62" s="17" t="inlineStr">
         <is>
-          <t>combinatorics, dp, math (Ôn lại: 330 ngày)</t>
+          <t>combinatorics, dp, math (Ôn lại: 329 ngày)</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
@@ -13068,7 +13362,7 @@
       </c>
       <c r="B95" s="17" t="inlineStr">
         <is>
-          <t>greedy, math, number theory (Ôn lại: 844 ngày)</t>
+          <t>greedy, math, number theory (Ôn lại: 843 ngày)</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
@@ -13148,7 +13442,7 @@
       </c>
       <c r="B99" s="17" t="inlineStr">
         <is>
-          <t>greedy, math (Ôn lại: 357 ngày)</t>
+          <t>greedy, math (Ôn lại: 356 ngày)</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
@@ -13168,7 +13462,7 @@
       </c>
       <c r="B100" s="17" t="inlineStr">
         <is>
-          <t>graphs, greedy, math (Ôn lại: 332 ngày)</t>
+          <t>graphs, greedy, math (Ôn lại: 331 ngày)</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
@@ -13755,7 +14049,7 @@
       </c>
       <c r="E23" s="17" t="inlineStr">
         <is>
-          <t>dp, sortings, string suffix structures (Ôn lại: 358 ngày)</t>
+          <t>dp, sortings, string suffix structures (Ôn lại: 357 ngày)</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -13863,12 +14157,12 @@
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>https://codeforces.com/problemset/problem/1991/E</t>
+          <t>https://codeforces.com/problemset/problem/1991/D</t>
         </is>
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>constructive algorithms, dfs and similar, games (Ôn lại: 809 ngày)</t>
+          <t>bitmasks, constructive algorithms, graphs (Ôn lại: 809 ngày)</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
@@ -13895,12 +14189,12 @@
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="16" t="inlineStr">
         <is>
-          <t>https://codeforces.com/problemset/problem/1991/D</t>
+          <t>https://codeforces.com/problemset/problem/1991/E</t>
         </is>
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>bitmasks, constructive algorithms, graphs (Ôn lại: 809 ngày)</t>
+          <t>constructive algorithms, dfs and similar, games (Ôn lại: 808 ngày)</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -14028,7 +14322,7 @@
       </c>
       <c r="B32" s="17" t="inlineStr">
         <is>
-          <t>constructive algorithms, dp (Ôn lại: 357 ngày)</t>
+          <t>constructive algorithms, dp (Ôn lại: 356 ngày)</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -16707,12 +17001,12 @@
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-11-20</t>
         </is>
       </c>
       <c r="I47" s="11" t="inlineStr">
         <is>
-          <t>330 ngày</t>
+          <t>329 ngày</t>
         </is>
       </c>
       <c r="J47" s="22" t="inlineStr">
@@ -17290,12 +17584,12 @@
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>2025-10-22</t>
+          <t>2025-10-23</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>358 ngày</t>
+          <t>357 ngày</t>
         </is>
       </c>
       <c r="J58" s="22" t="inlineStr">
@@ -17926,12 +18220,12 @@
       </c>
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2025-10-24</t>
         </is>
       </c>
       <c r="I70" s="11" t="inlineStr">
         <is>
-          <t>357 ngày</t>
+          <t>356 ngày</t>
         </is>
       </c>
       <c r="J70" s="22" t="inlineStr">
@@ -18615,12 +18909,12 @@
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>2025-11-17</t>
+          <t>2025-11-18</t>
         </is>
       </c>
       <c r="I83" s="11" t="inlineStr">
         <is>
-          <t>332 ngày</t>
+          <t>331 ngày</t>
         </is>
       </c>
       <c r="J83" s="22" t="inlineStr">
@@ -18640,17 +18934,17 @@
       </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>2041M</t>
+          <t>2041C</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>Selection Sort</t>
+          <t>Cube</t>
         </is>
       </c>
       <c r="D84" s="16" t="inlineStr">
         <is>
-          <t>https://codeforces.com/problemset/problem/2041/M</t>
+          <t>https://codeforces.com/problemset/problem/2041/C</t>
         </is>
       </c>
       <c r="E84" s="20" t="n">
@@ -18658,12 +18952,12 @@
       </c>
       <c r="F84" s="17" t="inlineStr">
         <is>
-          <t>Greedy &amp; Search</t>
+          <t>Graph Theory</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
         <is>
-          <t>binary search, data structures, greedy, two pointers</t>
+          <t>bitmasks, dfs and similar, dp</t>
         </is>
       </c>
       <c r="H84" s="6" t="inlineStr">
@@ -18693,17 +18987,17 @@
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>2041C</t>
+          <t>2041M</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Cube</t>
+          <t>Selection Sort</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>https://codeforces.com/problemset/problem/2041/C</t>
+          <t>https://codeforces.com/problemset/problem/2041/M</t>
         </is>
       </c>
       <c r="E85" s="20" t="n">
@@ -18711,22 +19005,22 @@
       </c>
       <c r="F85" s="17" t="inlineStr">
         <is>
-          <t>Graph Theory</t>
+          <t>Greedy &amp; Search</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr">
         <is>
-          <t>bitmasks, dfs and similar, dp</t>
+          <t>binary search, data structures, greedy, two pointers</t>
         </is>
       </c>
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-11-20</t>
         </is>
       </c>
       <c r="I85" s="11" t="inlineStr">
         <is>
-          <t>330 ngày</t>
+          <t>329 ngày</t>
         </is>
       </c>
       <c r="J85" s="22" t="inlineStr">
@@ -19092,12 +19386,12 @@
       </c>
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>2024-06-23</t>
+          <t>2024-06-24</t>
         </is>
       </c>
       <c r="I92" s="11" t="inlineStr">
         <is>
-          <t>844 ngày</t>
+          <t>843 ngày</t>
         </is>
       </c>
       <c r="J92" s="22" t="inlineStr">
@@ -19170,17 +19464,17 @@
       </c>
       <c r="B94" s="7" t="inlineStr">
         <is>
-          <t>1991E</t>
+          <t>1991D</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>Coloring Game</t>
+          <t>Prime XOR Coloring</t>
         </is>
       </c>
       <c r="D94" s="16" t="inlineStr">
         <is>
-          <t>https://codeforces.com/problemset/problem/1991/E</t>
+          <t>https://codeforces.com/problemset/problem/1991/D</t>
         </is>
       </c>
       <c r="E94" s="20" t="n">
@@ -19188,12 +19482,12 @@
       </c>
       <c r="F94" s="17" t="inlineStr">
         <is>
-          <t>Graph Theory</t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
-          <t>constructive algorithms, dfs and similar, games, graphs, greedy</t>
+          <t>bitmasks, constructive algorithms, graphs, greedy, math</t>
         </is>
       </c>
       <c r="H94" s="6" t="inlineStr">
@@ -19223,17 +19517,17 @@
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>1991D</t>
+          <t>1991E</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>Prime XOR Coloring</t>
+          <t>Coloring Game</t>
         </is>
       </c>
       <c r="D95" s="16" t="inlineStr">
         <is>
-          <t>https://codeforces.com/problemset/problem/1991/D</t>
+          <t>https://codeforces.com/problemset/problem/1991/E</t>
         </is>
       </c>
       <c r="E95" s="20" t="n">
@@ -19241,22 +19535,22 @@
       </c>
       <c r="F95" s="17" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>Graph Theory</t>
         </is>
       </c>
       <c r="G95" s="3" t="inlineStr">
         <is>
-          <t>bitmasks, constructive algorithms, graphs, greedy, math</t>
+          <t>constructive algorithms, dfs and similar, games, graphs, greedy</t>
         </is>
       </c>
       <c r="H95" s="6" t="inlineStr">
         <is>
-          <t>2024-07-28</t>
+          <t>2024-07-29</t>
         </is>
       </c>
       <c r="I95" s="11" t="inlineStr">
         <is>
-          <t>809 ngày</t>
+          <t>808 ngày</t>
         </is>
       </c>
       <c r="J95" s="22" t="inlineStr">
@@ -19569,12 +19863,12 @@
       </c>
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2025-10-24</t>
         </is>
       </c>
       <c r="I101" s="11" t="inlineStr">
         <is>
-          <t>357 ngày</t>
+          <t>356 ngày</t>
         </is>
       </c>
       <c r="J101" s="22" t="inlineStr">
@@ -20258,12 +20552,12 @@
       </c>
       <c r="H114" s="6" t="inlineStr">
         <is>
-          <t>2025-10-22</t>
+          <t>2025-10-23</t>
         </is>
       </c>
       <c r="I114" s="11" t="inlineStr">
         <is>
-          <t>358 ngày</t>
+          <t>357 ngày</t>
         </is>
       </c>
       <c r="J114" s="22" t="inlineStr">
@@ -20625,12 +20919,12 @@
       </c>
       <c r="H121" s="6" t="inlineStr">
         <is>
-          <t>2024-06-23</t>
+          <t>2024-06-24</t>
         </is>
       </c>
       <c r="I121" s="11" t="inlineStr">
         <is>
-          <t>844 ngày</t>
+          <t>843 ngày</t>
         </is>
       </c>
       <c r="J121" s="10" t="inlineStr">
@@ -20890,12 +21184,12 @@
       </c>
       <c r="H126" s="6" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2025-10-24</t>
         </is>
       </c>
       <c r="I126" s="11" t="inlineStr">
         <is>
-          <t>357 ngày</t>
+          <t>356 ngày</t>
         </is>
       </c>
       <c r="J126" s="10" t="inlineStr">
@@ -21420,12 +21714,12 @@
       </c>
       <c r="H136" s="6" t="inlineStr">
         <is>
-          <t>2025-11-17</t>
+          <t>2025-11-18</t>
         </is>
       </c>
       <c r="I136" s="11" t="inlineStr">
         <is>
-          <t>332 ngày</t>
+          <t>331 ngày</t>
         </is>
       </c>
       <c r="J136" s="10" t="inlineStr">

</xml_diff>